<commit_message>
Adiciona gerador de relatórios (PDF/planilha) e relatórios de sushi e pizzarias
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DezMuieR4YXnuzPVtL38Eh
</commit_message>
<xml_diff>
--- a/delivery_joinville/sushi_joinville_google_places.xlsx
+++ b/delivery_joinville/sushi_joinville_google_places.xlsx
@@ -7,12 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sushi e japonesa" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sushi, japonesa, oriental e pok" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Outros resultados" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Notas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sushi e japonesa'!$A$1:$L$102</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sushi, japonesa, oriental e pok'!$A$1:$L$102</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Outros resultados'!$A$1:$L$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8410,21 +8410,21 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Termos buscados: "sushi", "comida japonesa", "temakeria", "poke" + Joinville, em 16 regiões da cidade.</t>
+          <t>Termos buscados: "sushi", "comida japonesa", "temakeria" e "poke" + Joinville, em 16 regiões da cidade.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Aba "Sushi e japonesa": resultados cujo tipo no Google ou nome indica sushi/japonesa/oriental/poke.</t>
+          <t>Aba "Sushi, japonesa, oriental e poke": resultados cujo tipo no Google ou nome indica essa categoria.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Aba "Outros resultados": apareceram na busca (podem ter sushi no cardápio), mas não são restaurantes japoneses.</t>
+          <t>Aba "Outros resultados": apareceram na busca, mas o cadastro no Google indica outra categoria.</t>
         </is>
       </c>
     </row>

</xml_diff>